<commit_message>
Update slime art, monster groups and random spawn design
</commit_message>
<xml_diff>
--- a/Excel/Dialogue.xlsx
+++ b/Excel/Dialogue.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="480">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="505" uniqueCount="505">
   <si>
     <t/>
   </si>
@@ -1455,6 +1455,81 @@
   </si>
   <si>
     <t>第一次上台</t>
+  </si>
+  <si>
+    <t>老板，近来路上的怪物越聚越多，要在失落大陆上经营酒馆，不多备两件实用的防具可护不住周全。</t>
+  </si>
+  <si>
+    <t>老板，镇外的怪物最近成群出现，光靠粗木棒和匕首可应付不来。我想挑一把结实顺手的铁剑，接战斗委托时好开出一条生路。</t>
+  </si>
+  <si>
+    <t>镇上要是有战斗悬赏就贴出来吧。我得先在板前摸清那群怪物的数量和聚集地点，算清胜算，再决定接不接。</t>
+  </si>
+  <si>
+    <t>这条情报说的是：{到来时间}，{地点}出现了一群{怪物名}，共有{怪物数量}只。</t>
+  </si>
+  <si>
+    <t>若想在它们袭击商道前清除这群怪物，就去酒馆的悬赏板立一份悬赏，自会有贪求赏金的佣兵前去揭榜。</t>
+  </si>
+  <si>
+    <t>那群怪物的讨伐悬赏，我已经正式发布在悬赏栏上了。</t>
+  </si>
+  <si>
+    <t>你买下的消息确凿无误。就在{到来时间}，{地点}出现了一群{怪物名}，共有{怪物数量}只。</t>
+  </si>
+  <si>
+    <t>采买和运货的人都得经过那一带。绕远路费工夫，硬着头皮走又提心吊胆，这麻烦早晚得解决。</t>
+  </si>
+  <si>
+    <t>要是挂出悬赏，真有人敢接这趟差事吗？成群的怪物有多难对付，大伙心里都有数。</t>
+  </si>
+  <si>
+    <t>我明白了。既然这群怪物挡着大伙的路，这份悬赏单，我得找羊皮纸好好写写。</t>
+  </si>
+  <si>
+    <t>悬赏已发布：清除{地点}的这群{怪物名}。</t>
+  </si>
+  <si>
+    <t>悬赏已完成，绑定怪物组已全部清除，报酬已结算。</t>
+  </si>
+  <si>
+    <t>这群怪物已被其他人全部清除，无须再为它们发布悬赏。</t>
+  </si>
+  <si>
+    <t>{地点}那桩悬赏结了。那群{怪物名}已经全部清除，赏金也结清了。</t>
+  </si>
+  <si>
+    <t>呼……总算能松口气。虽说以后未必一直太平，但起码今天经过那里的人能安心走路了。</t>
+  </si>
+  <si>
+    <t>去{地点}接赏的那位……没能活着回来。悬赏没办成，人折在那里了。</t>
+  </si>
+  <si>
+    <t>……是么。我只当那群怪物会拖慢几趟脚程，没想到真搭进去一条命。买卖归买卖，这消息听着堵心。</t>
+  </si>
+  <si>
+    <t>路上的怪物群</t>
+  </si>
+  <si>
+    <t>前段读完后有新怪物组到来，玩家向绑定诗人成功购买该组情报后播放；购买时组内至少一只存活且无玩家针对该组的悬赏。未成交不播详情。</t>
+  </si>
+  <si>
+    <t>针对上一段绑定的怪物组实例发布悬赏成功后，与绑定诗人交谈；读取实际发布记录，不由本段代发悬赏。</t>
+  </si>
+  <si>
+    <t>任一种已解锁怪物组在随机场地实际生成，玩家向知情诗人成功购买该组情报后播放；monster_id=0，不限制怪种与场地。购买时组内至少一只存活且无对应悬赏。与main07_02命中同次购买时只播本段并同步进度。</t>
+  </si>
+  <si>
+    <t>本次绑定怪物组的悬赏发布成功后显示系统提示；目标数量取发布时存活成员数。前段未读完时保留记录，待其读完再播。</t>
+  </si>
+  <si>
+    <t>购买情报后、玩家发布悬赏前，同一怪物组的全部成员已被其他人清除；前段读完后显示，不再进入发布分支。</t>
+  </si>
+  <si>
+    <t>Ex01_03已读后，与原出售情报的诗人交谈；沿用同一怪物组实例和悬赏的成功、结算记录。诗人暂离则等待，死亡或永久离开则结束；本段读完结束成功分支。</t>
+  </si>
+  <si>
+    <t>悬赏已完成，目标怪物已全部清除，报酬已结算。</t>
   </si>
 </sst>
 </file>
@@ -1532,7 +1607,7 @@
     <xf numFmtId="300" fontId="5" fillId="0" borderId="1" xfId="0"/>
     <xf numFmtId="300" fontId="5" fillId="2" borderId="1" xfId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1553,6 +1628,12 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="300" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2507,8 +2588,8 @@
       <c r="E35" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F35" s="5" t="s">
-        <v>116</v>
+      <c r="F35" s="8" t="s">
+        <v>480</v>
       </c>
       <c r="G35" s="5">
         <v>2</v>
@@ -2528,7 +2609,7 @@
       <c r="E36" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F36" s="5" t="s">
+      <c r="F36" s="8" t="s">
         <v>118</v>
       </c>
       <c r="G36" s="5">
@@ -2549,7 +2630,7 @@
       <c r="E37" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F37" s="5" t="s">
+      <c r="F37" s="8" t="s">
         <v>121</v>
       </c>
       <c r="G37" s="5">
@@ -2570,7 +2651,7 @@
       <c r="E38" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F38" s="5" t="s">
+      <c r="F38" s="8" t="s">
         <v>123</v>
       </c>
       <c r="G38" s="5">
@@ -2591,7 +2672,7 @@
       <c r="E39" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F39" s="5" t="s">
+      <c r="F39" s="8" t="s">
         <v>126</v>
       </c>
       <c r="G39" s="5">
@@ -2612,7 +2693,7 @@
       <c r="E40" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F40" s="5" t="s">
+      <c r="F40" s="8" t="s">
         <v>128</v>
       </c>
       <c r="G40" s="5">
@@ -2633,7 +2714,7 @@
       <c r="E41" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F41" s="5" t="s">
+      <c r="F41" s="8" t="s">
         <v>131</v>
       </c>
       <c r="G41" s="5">
@@ -2654,7 +2735,7 @@
       <c r="E42" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F42" s="5" t="s">
+      <c r="F42" s="8" t="s">
         <v>133</v>
       </c>
       <c r="G42" s="5">
@@ -2675,7 +2756,7 @@
       <c r="E43" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="F43" s="5" t="s">
+      <c r="F43" s="8" t="s">
         <v>136</v>
       </c>
       <c r="G43" s="5">
@@ -2696,7 +2777,7 @@
       <c r="E44" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F44" s="5" t="s">
+      <c r="F44" s="8" t="s">
         <v>138</v>
       </c>
       <c r="G44" s="5">
@@ -2717,7 +2798,7 @@
       <c r="E45" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F45" s="5" t="s">
+      <c r="F45" s="8" t="s">
         <v>141</v>
       </c>
       <c r="G45" s="5">
@@ -2738,7 +2819,7 @@
       <c r="E46" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F46" s="5" t="s">
+      <c r="F46" s="8" t="s">
         <v>143</v>
       </c>
       <c r="G46" s="5">
@@ -2759,7 +2840,7 @@
       <c r="E47" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F47" s="5" t="s">
+      <c r="F47" s="8" t="s">
         <v>146</v>
       </c>
       <c r="G47" s="5">
@@ -2780,7 +2861,7 @@
       <c r="E48" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F48" s="5" t="s">
+      <c r="F48" s="8" t="s">
         <v>148</v>
       </c>
       <c r="G48" s="5">
@@ -2801,7 +2882,7 @@
       <c r="E49" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F49" s="5" t="s">
+      <c r="F49" s="8" t="s">
         <v>151</v>
       </c>
       <c r="G49" s="5">
@@ -2822,7 +2903,7 @@
       <c r="E50" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F50" s="5" t="s">
+      <c r="F50" s="8" t="s">
         <v>153</v>
       </c>
       <c r="G50" s="5">
@@ -2843,7 +2924,7 @@
       <c r="E51" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F51" s="5" t="s">
+      <c r="F51" s="8" t="s">
         <v>156</v>
       </c>
       <c r="G51" s="5">
@@ -2864,7 +2945,7 @@
       <c r="E52" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F52" s="5" t="s">
+      <c r="F52" s="8" t="s">
         <v>158</v>
       </c>
       <c r="G52" s="5">
@@ -2885,8 +2966,8 @@
       <c r="E53" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F53" s="5" t="s">
-        <v>161</v>
+      <c r="F53" s="8" t="s">
+        <v>481</v>
       </c>
       <c r="G53" s="5">
         <v>5</v>
@@ -2906,7 +2987,7 @@
       <c r="E54" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F54" s="5" t="s">
+      <c r="F54" s="8" t="s">
         <v>163</v>
       </c>
       <c r="G54" s="5">
@@ -2927,7 +3008,7 @@
       <c r="E55" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F55" s="5" t="s">
+      <c r="F55" s="8" t="s">
         <v>166</v>
       </c>
       <c r="G55" s="5">
@@ -2948,8 +3029,8 @@
       <c r="E56" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F56" s="5" t="s">
-        <v>168</v>
+      <c r="F56" s="8" t="s">
+        <v>482</v>
       </c>
       <c r="G56" s="5">
         <v>5</v>
@@ -2969,7 +3050,7 @@
       <c r="E57" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F57" s="5" t="s">
+      <c r="F57" s="8" t="s">
         <v>171</v>
       </c>
       <c r="G57" s="5">
@@ -2990,7 +3071,7 @@
       <c r="E58" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F58" s="5" t="s">
+      <c r="F58" s="8" t="s">
         <v>173</v>
       </c>
       <c r="G58" s="5">
@@ -3011,7 +3092,7 @@
       <c r="E59" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="F59" s="5" t="s">
+      <c r="F59" s="8" t="s">
         <v>177</v>
       </c>
       <c r="G59" s="5">
@@ -3032,7 +3113,7 @@
       <c r="E60" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F60" s="5" t="s">
+      <c r="F60" s="8" t="s">
         <v>180</v>
       </c>
       <c r="G60" s="5">
@@ -3053,7 +3134,7 @@
       <c r="E61" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F61" s="5" t="s">
+      <c r="F61" s="8" t="s">
         <v>182</v>
       </c>
       <c r="G61" s="5">
@@ -3074,7 +3155,7 @@
       <c r="E62" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F62" s="5" t="s">
+      <c r="F62" s="8" t="s">
         <v>185</v>
       </c>
       <c r="G62" s="5">
@@ -3095,7 +3176,7 @@
       <c r="E63" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F63" s="5" t="s">
+      <c r="F63" s="8" t="s">
         <v>187</v>
       </c>
       <c r="G63" s="5">
@@ -3116,7 +3197,7 @@
       <c r="E64" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F64" s="5" t="s">
+      <c r="F64" s="8" t="s">
         <v>190</v>
       </c>
       <c r="G64" s="5">
@@ -3137,7 +3218,7 @@
       <c r="E65" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F65" s="5" t="s">
+      <c r="F65" s="8" t="s">
         <v>192</v>
       </c>
       <c r="G65" s="5">
@@ -3158,7 +3239,7 @@
       <c r="E66" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F66" s="5" t="s">
+      <c r="F66" s="8" t="s">
         <v>195</v>
       </c>
       <c r="G66" s="5">
@@ -3179,7 +3260,7 @@
       <c r="E67" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F67" s="5" t="s">
+      <c r="F67" s="8" t="s">
         <v>197</v>
       </c>
       <c r="G67" s="5">
@@ -3200,8 +3281,8 @@
       <c r="E68" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F68" s="5" t="s">
-        <v>200</v>
+      <c r="F68" s="8" t="s">
+        <v>483</v>
       </c>
       <c r="G68" s="5">
         <v>7</v>
@@ -3221,8 +3302,8 @@
       <c r="E69" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F69" s="5" t="s">
-        <v>202</v>
+      <c r="F69" s="8" t="s">
+        <v>484</v>
       </c>
       <c r="G69" s="5">
         <v>7</v>
@@ -3242,8 +3323,8 @@
       <c r="E70" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="F70" s="5" t="s">
-        <v>205</v>
+      <c r="F70" s="8" t="s">
+        <v>485</v>
       </c>
       <c r="G70" s="5">
         <v>7</v>
@@ -3263,7 +3344,7 @@
       <c r="E71" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F71" s="5" t="s">
+      <c r="F71" s="8" t="s">
         <v>207</v>
       </c>
       <c r="G71" s="5">
@@ -3284,8 +3365,8 @@
       <c r="E72" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F72" s="5" t="s">
-        <v>210</v>
+      <c r="F72" s="8" t="s">
+        <v>486</v>
       </c>
       <c r="G72" s="5">
         <v>7</v>
@@ -3305,8 +3386,8 @@
       <c r="E73" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F73" s="5" t="s">
-        <v>212</v>
+      <c r="F73" s="8" t="s">
+        <v>487</v>
       </c>
       <c r="G73" s="5">
         <v>7</v>
@@ -3326,8 +3407,8 @@
       <c r="E74" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="F74" s="5" t="s">
-        <v>214</v>
+      <c r="F74" s="8" t="s">
+        <v>488</v>
       </c>
       <c r="G74" s="5">
         <v>7</v>
@@ -3347,7 +3428,7 @@
       <c r="E75" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F75" s="5" t="s">
+      <c r="F75" s="8" t="s">
         <v>216</v>
       </c>
       <c r="G75" s="5">
@@ -3368,8 +3449,8 @@
       <c r="E76" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="F76" s="5" t="s">
-        <v>218</v>
+      <c r="F76" s="8" t="s">
+        <v>489</v>
       </c>
       <c r="G76" s="5">
         <v>7</v>
@@ -3389,8 +3470,8 @@
       <c r="E77" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="F77" s="5" t="s">
-        <v>221</v>
+      <c r="F77" s="8" t="s">
+        <v>490</v>
       </c>
       <c r="G77" s="5">
         <v>0</v>
@@ -3410,8 +3491,8 @@
       <c r="E78" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="F78" s="5" t="s">
-        <v>224</v>
+      <c r="F78" s="8" t="s">
+        <v>504</v>
       </c>
       <c r="G78" s="5">
         <v>0</v>
@@ -3431,7 +3512,7 @@
       <c r="E79" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="F79" s="5" t="s">
+      <c r="F79" s="8" t="s">
         <v>227</v>
       </c>
       <c r="G79" s="5">
@@ -3452,8 +3533,8 @@
       <c r="E80" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="F80" s="5" t="s">
-        <v>230</v>
+      <c r="F80" s="8" t="s">
+        <v>492</v>
       </c>
       <c r="G80" s="5">
         <v>0</v>
@@ -3473,7 +3554,7 @@
       <c r="E81" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="F81" s="5" t="s">
+      <c r="F81" s="8" t="s">
         <v>233</v>
       </c>
       <c r="G81" s="5">
@@ -3494,8 +3575,8 @@
       <c r="E82" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="F82" s="5" t="s">
-        <v>236</v>
+      <c r="F82" s="8" t="s">
+        <v>493</v>
       </c>
       <c r="G82" s="5">
         <v>7</v>
@@ -3515,8 +3596,8 @@
       <c r="E83" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F83" s="5" t="s">
-        <v>238</v>
+      <c r="F83" s="8" t="s">
+        <v>494</v>
       </c>
       <c r="G83" s="5">
         <v>7</v>
@@ -3536,7 +3617,7 @@
       <c r="E84" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="F84" s="5" t="s">
+      <c r="F84" s="8" t="s">
         <v>240</v>
       </c>
       <c r="G84" s="5">
@@ -3557,8 +3638,8 @@
       <c r="E85" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="F85" s="5" t="s">
-        <v>243</v>
+      <c r="F85" s="8" t="s">
+        <v>495</v>
       </c>
       <c r="G85" s="5">
         <v>7</v>
@@ -3578,8 +3659,8 @@
       <c r="E86" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F86" s="5" t="s">
-        <v>245</v>
+      <c r="F86" s="8" t="s">
+        <v>496</v>
       </c>
       <c r="G86" s="5">
         <v>7</v>
@@ -6127,8 +6208,8 @@
       <c r="M49" s="7">
         <v>1000</v>
       </c>
-      <c r="N49" s="7" t="s">
-        <v>441</v>
+      <c r="N49" s="9" t="s">
+        <v>498</v>
       </c>
     </row>
     <row r="50" spans="1:14" ht="42" customHeight="1">
@@ -6169,8 +6250,8 @@
       <c r="M50" s="7">
         <v>1000</v>
       </c>
-      <c r="N50" s="7" t="s">
-        <v>443</v>
+      <c r="N50" s="9" t="s">
+        <v>499</v>
       </c>
     </row>
     <row r="51" spans="1:14" ht="42" customHeight="1">
@@ -6181,8 +6262,8 @@
       <c r="C51" s="5" t="s">
         <v>444</v>
       </c>
-      <c r="D51" s="5" t="s">
-        <v>445</v>
+      <c r="D51" s="8" t="s">
+        <v>497</v>
       </c>
       <c r="E51" s="5" t="s">
         <v>446</v>
@@ -6197,8 +6278,8 @@
       <c r="I51" s="5">
         <v>0</v>
       </c>
-      <c r="J51" s="7">
-        <v>3</v>
+      <c r="J51" s="9">
+        <v>0</v>
       </c>
       <c r="K51" s="7">
         <v>0</v>
@@ -6209,8 +6290,8 @@
       <c r="M51" s="7">
         <v>1000</v>
       </c>
-      <c r="N51" s="7" t="s">
-        <v>447</v>
+      <c r="N51" s="9" t="s">
+        <v>500</v>
       </c>
     </row>
     <row r="52" spans="1:14" ht="42" customHeight="1">
@@ -6221,8 +6302,8 @@
       <c r="C52" s="5" t="s">
         <v>444</v>
       </c>
-      <c r="D52" s="5" t="s">
-        <v>445</v>
+      <c r="D52" s="8" t="s">
+        <v>497</v>
       </c>
       <c r="E52" s="5" t="s">
         <v>446</v>
@@ -6251,8 +6332,8 @@
       <c r="M52" s="7">
         <v>1000</v>
       </c>
-      <c r="N52" s="7" t="s">
-        <v>449</v>
+      <c r="N52" s="9" t="s">
+        <v>501</v>
       </c>
     </row>
     <row r="53" spans="1:14" ht="42" customHeight="1">
@@ -6263,8 +6344,8 @@
       <c r="C53" s="5" t="s">
         <v>444</v>
       </c>
-      <c r="D53" s="5" t="s">
-        <v>445</v>
+      <c r="D53" s="8" t="s">
+        <v>497</v>
       </c>
       <c r="E53" s="5" t="s">
         <v>446</v>
@@ -6293,7 +6374,7 @@
       <c r="M53" s="7">
         <v>1000</v>
       </c>
-      <c r="N53" s="7" t="s">
+      <c r="N53" s="9" t="s">
         <v>451</v>
       </c>
     </row>
@@ -6305,8 +6386,8 @@
       <c r="C54" s="5" t="s">
         <v>444</v>
       </c>
-      <c r="D54" s="5" t="s">
-        <v>445</v>
+      <c r="D54" s="8" t="s">
+        <v>497</v>
       </c>
       <c r="E54" s="5" t="s">
         <v>446</v>
@@ -6335,7 +6416,7 @@
       <c r="M54" s="7">
         <v>1000</v>
       </c>
-      <c r="N54" s="7" t="s">
+      <c r="N54" s="9" t="s">
         <v>453</v>
       </c>
     </row>
@@ -6347,8 +6428,8 @@
       <c r="C55" s="5" t="s">
         <v>444</v>
       </c>
-      <c r="D55" s="5" t="s">
-        <v>445</v>
+      <c r="D55" s="8" t="s">
+        <v>497</v>
       </c>
       <c r="E55" s="5" t="s">
         <v>446</v>
@@ -6377,8 +6458,8 @@
       <c r="M55" s="7">
         <v>1000</v>
       </c>
-      <c r="N55" s="7" t="s">
-        <v>455</v>
+      <c r="N55" s="9" t="s">
+        <v>502</v>
       </c>
     </row>
     <row r="56" spans="1:14" ht="42" customHeight="1">
@@ -6389,8 +6470,8 @@
       <c r="C56" s="5" t="s">
         <v>444</v>
       </c>
-      <c r="D56" s="5" t="s">
-        <v>445</v>
+      <c r="D56" s="8" t="s">
+        <v>497</v>
       </c>
       <c r="E56" s="5" t="s">
         <v>446</v>
@@ -6419,7 +6500,7 @@
       <c r="M56" s="7">
         <v>1000</v>
       </c>
-      <c r="N56" s="7" t="s">
+      <c r="N56" s="9" t="s">
         <v>457</v>
       </c>
     </row>
@@ -6431,8 +6512,8 @@
       <c r="C57" s="5" t="s">
         <v>444</v>
       </c>
-      <c r="D57" s="5" t="s">
-        <v>445</v>
+      <c r="D57" s="8" t="s">
+        <v>497</v>
       </c>
       <c r="E57" s="5" t="s">
         <v>446</v>
@@ -6461,8 +6542,8 @@
       <c r="M57" s="7">
         <v>1000</v>
       </c>
-      <c r="N57" s="7" t="s">
-        <v>459</v>
+      <c r="N57" s="9" t="s">
+        <v>503</v>
       </c>
     </row>
     <row r="58" spans="1:14" ht="42" customHeight="1">
@@ -6473,8 +6554,8 @@
       <c r="C58" s="5" t="s">
         <v>444</v>
       </c>
-      <c r="D58" s="5" t="s">
-        <v>445</v>
+      <c r="D58" s="8" t="s">
+        <v>497</v>
       </c>
       <c r="E58" s="5" t="s">
         <v>446</v>
@@ -6503,7 +6584,7 @@
       <c r="M58" s="7">
         <v>1000</v>
       </c>
-      <c r="N58" s="7" t="s">
+      <c r="N58" s="9" t="s">
         <v>461</v>
       </c>
     </row>

</xml_diff>